<commit_message>
reports/cnn: refresh the combined22 results workbook
</commit_message>
<xml_diff>
--- a/reports/cnn/ContactLensDefectResults_combined22.xlsx
+++ b/reports/cnn/ContactLensDefectResults_combined22.xlsx
@@ -1,27 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\02-SSA\fmd-analysis\reports\cnn\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fmd-analysis\reports\cnn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA376C1D-9211-4211-B38D-F7D9BBDA9820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EAEC3E7-3209-43F1-B0BE-43F9E8EF275D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Comparison vs teammate" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -381,10 +376,19 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -393,15 +397,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -716,63 +711,63 @@
     <col min="6" max="27" width="7" customWidth="1"/>
     <col min="28" max="28" width="14" customWidth="1"/>
     <col min="29" max="29" width="16" customWidth="1"/>
-    <col min="30" max="30" width="20.5703125" style="13" customWidth="1"/>
+    <col min="30" max="30" width="20.5703125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="10"/>
-      <c r="AB1" s="5" t="s">
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AC1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AD1" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
@@ -839,15 +834,15 @@
       <c r="AA2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AB2" s="6"/>
-      <c r="AC2" s="6"/>
-      <c r="AD2" s="12"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="8"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -931,7 +926,7 @@
       <c r="AC3" s="3">
         <v>0.67</v>
       </c>
-      <c r="AD3" s="13" t="s">
+      <c r="AD3" s="5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -939,7 +934,7 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="3" t="s">
         <v>33</v>
       </c>
@@ -1021,7 +1016,7 @@
       <c r="AC4" s="3">
         <v>1.28</v>
       </c>
-      <c r="AD4" s="13" t="s">
+      <c r="AD4" s="5" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1029,7 +1024,7 @@
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="11"/>
       <c r="C5" s="3" t="s">
         <v>35</v>
       </c>
@@ -1111,7 +1106,7 @@
       <c r="AC5" s="3">
         <v>1.75</v>
       </c>
-      <c r="AD5" s="13" t="s">
+      <c r="AD5" s="5" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1119,7 +1114,7 @@
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="8"/>
+      <c r="B6" s="11"/>
       <c r="C6" s="3" t="s">
         <v>37</v>
       </c>
@@ -1201,7 +1196,7 @@
       <c r="AC6" s="3">
         <v>1.51</v>
       </c>
-      <c r="AD6" s="13" t="s">
+      <c r="AD6" s="5" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1209,8 +1204,8 @@
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="14" t="s">
+      <c r="B7" s="11"/>
+      <c r="C7" s="6" t="s">
         <v>39</v>
       </c>
       <c r="D7" s="3">
@@ -1291,7 +1286,7 @@
       <c r="AC7" s="3">
         <v>1.76</v>
       </c>
-      <c r="AD7" s="13" t="s">
+      <c r="AD7" s="5" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1299,8 +1294,8 @@
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="14" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="D8" s="3">
@@ -1381,7 +1376,7 @@
       <c r="AC8" s="3">
         <v>2.12</v>
       </c>
-      <c r="AD8" s="13" t="s">
+      <c r="AD8" s="5" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1431,131 +1426,131 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="11"/>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="14"/>
+      <c r="G1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="5" t="s">
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="5" t="s">
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="5" t="s">
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="5" t="s">
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="5" t="s">
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="5" t="s">
+      <c r="W1" s="14"/>
+      <c r="X1" s="14"/>
+      <c r="Y1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Z1" s="11"/>
-      <c r="AA1" s="11"/>
-      <c r="AB1" s="5" t="s">
+      <c r="Z1" s="14"/>
+      <c r="AA1" s="14"/>
+      <c r="AB1" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="AC1" s="11"/>
-      <c r="AD1" s="11"/>
-      <c r="AE1" s="5" t="s">
+      <c r="AC1" s="14"/>
+      <c r="AD1" s="14"/>
+      <c r="AE1" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="AF1" s="11"/>
-      <c r="AG1" s="11"/>
-      <c r="AH1" s="5" t="s">
+      <c r="AF1" s="14"/>
+      <c r="AG1" s="14"/>
+      <c r="AH1" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="AI1" s="11"/>
-      <c r="AJ1" s="11"/>
-      <c r="AK1" s="5" t="s">
+      <c r="AI1" s="14"/>
+      <c r="AJ1" s="14"/>
+      <c r="AK1" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="AL1" s="11"/>
-      <c r="AM1" s="11"/>
-      <c r="AN1" s="5" t="s">
+      <c r="AL1" s="14"/>
+      <c r="AM1" s="14"/>
+      <c r="AN1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="AO1" s="11"/>
-      <c r="AP1" s="11"/>
-      <c r="AQ1" s="5" t="s">
+      <c r="AO1" s="14"/>
+      <c r="AP1" s="14"/>
+      <c r="AQ1" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AR1" s="11"/>
-      <c r="AS1" s="11"/>
-      <c r="AT1" s="5" t="s">
+      <c r="AR1" s="14"/>
+      <c r="AS1" s="14"/>
+      <c r="AT1" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="AU1" s="11"/>
-      <c r="AV1" s="11"/>
-      <c r="AW1" s="5" t="s">
+      <c r="AU1" s="14"/>
+      <c r="AV1" s="14"/>
+      <c r="AW1" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="AX1" s="11"/>
-      <c r="AY1" s="11"/>
-      <c r="AZ1" s="5" t="s">
+      <c r="AX1" s="14"/>
+      <c r="AY1" s="14"/>
+      <c r="AZ1" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="BA1" s="11"/>
-      <c r="BB1" s="11"/>
-      <c r="BC1" s="5" t="s">
+      <c r="BA1" s="14"/>
+      <c r="BB1" s="14"/>
+      <c r="BC1" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="BD1" s="11"/>
-      <c r="BE1" s="11"/>
-      <c r="BF1" s="5" t="s">
+      <c r="BD1" s="14"/>
+      <c r="BE1" s="14"/>
+      <c r="BF1" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="BG1" s="11"/>
-      <c r="BH1" s="11"/>
-      <c r="BI1" s="5" t="s">
+      <c r="BG1" s="14"/>
+      <c r="BH1" s="14"/>
+      <c r="BI1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="BJ1" s="11"/>
-      <c r="BK1" s="11"/>
-      <c r="BL1" s="5" t="s">
+      <c r="BJ1" s="14"/>
+      <c r="BK1" s="14"/>
+      <c r="BL1" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="BM1" s="11"/>
-      <c r="BN1" s="11"/>
-      <c r="BO1" s="5" t="s">
+      <c r="BM1" s="14"/>
+      <c r="BN1" s="14"/>
+      <c r="BO1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="11"/>
-      <c r="BQ1" s="11"/>
-      <c r="BR1" s="5" t="s">
+      <c r="BP1" s="14"/>
+      <c r="BQ1" s="14"/>
+      <c r="BR1" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="BS1" s="11"/>
-      <c r="BT1" s="11"/>
+      <c r="BS1" s="14"/>
+      <c r="BT1" s="14"/>
     </row>
     <row r="2" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
+      <c r="A2" s="14"/>
       <c r="B2" s="2" t="s">
         <v>68</v>
       </c>
@@ -3105,13 +3100,7 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="BR1:BT1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="V1:X1"/>
-    <mergeCell ref="AB1:AD1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="AT1:AV1"/>
-    <mergeCell ref="BF1:BH1"/>
+    <mergeCell ref="E1:F1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="P1:R1"/>
@@ -3128,8 +3117,14 @@
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="AE1:AG1"/>
+    <mergeCell ref="BR1:BT1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="V1:X1"/>
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="AT1:AV1"/>
+    <mergeCell ref="BF1:BH1"/>
     <mergeCell ref="AK1:AM1"/>
-    <mergeCell ref="E1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:B8">
     <cfRule type="colorScale" priority="2">

</xml_diff>